<commit_message>
docs: add presentation and demo recording
</commit_message>
<xml_diff>
--- a/산출물/COG_관리기준표.xlsx
+++ b/산출물/COG_관리기준표.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" r:id="R8095c6c967d44e4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI_관리기준" sheetId="2" r:id="R4c4ba37a85b943dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="변수_관리기준" sheetId="3" r:id="R1b13f1456c774840"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외_이벤트" sheetId="4" r:id="Raeffe2ca505d48c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" r:id="Rc2dc37635b1c44f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI_관리기준" sheetId="2" r:id="R36902373e2f64e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="변수_관리기준" sheetId="3" r:id="Re2590b314e514b94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외_이벤트" sheetId="4" r:id="Rac3800b679fc4576"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -597,6 +597,8 @@
       <x:c r="J2" s="33"/>
       <x:c r="K2" s="33"/>
       <x:c r="L2" s="33"/>
+      <x:c r="M2"/>
+      <x:c r="N2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="14" t="str">
@@ -807,7 +809,7 @@
       <x:c r="B8" s="38" t="str">
         <x:v>약품 A 원단위</x:v>
       </x:c>
-      <x:c r="C8" s="38" t="str"/>
+      <x:c r="C8" s="38"/>
       <x:c r="D8" s="38" t="str">
         <x:v>낮을수록 좋음</x:v>
       </x:c>
@@ -843,7 +845,7 @@
       <x:c r="B9" s="38" t="str">
         <x:v>약품 B 원단위</x:v>
       </x:c>
-      <x:c r="C9" s="38" t="str"/>
+      <x:c r="C9" s="38"/>
       <x:c r="D9" s="38" t="str">
         <x:v>낮을수록 좋음</x:v>
       </x:c>
@@ -880,31 +882,29 @@
         <x:v>스팀 전체 사용량</x:v>
       </x:c>
       <x:c r="C10" s="38" t="str">
-        <x:v>ton/일</x:v>
+        <x:v>t/h</x:v>
       </x:c>
       <x:c r="D10" s="38" t="str">
         <x:v>낮을수록 좋음</x:v>
       </x:c>
       <x:c r="E10" s="38" t="n">
-        <x:v>36.2784</x:v>
+        <x:v>15.116216592776157</x:v>
       </x:c>
       <x:c r="F10" s="38" t="n">
-        <x:v>36.6412</x:v>
+        <x:v>15.116216592776157</x:v>
       </x:c>
       <x:c r="G10" s="38"/>
       <x:c r="H10" s="38"/>
-      <x:c r="I10" s="38" t="n">
-        <x:v>36.7467</x:v>
-      </x:c>
+      <x:c r="I10" s="38"/>
       <x:c r="J10" s="38" t="n">
-        <x:v>36.9303</x:v>
-      </x:c>
-      <x:c r="K10" s="38"/>
-      <x:c r="L10" s="38" t="n">
-        <x:v>36.9303</x:v>
-      </x:c>
-      <x:c r="M10" s="27" t="str">
-        <x:v>주의: 정상 P95~P99; 이상: P99 초과</x:v>
+        <x:v>15.777943912865863</x:v>
+      </x:c>
+      <x:c r="K10" s="38" t="n">
+        <x:v>15.890471962477498</x:v>
+      </x:c>
+      <x:c r="L10" s="38"/>
+      <x:c r="M10" s="27" t="n">
+        <x:v>15.890471962477498</x:v>
       </x:c>
       <x:c r="N10" s="28" t="str">
         <x:v>P95 이하</x:v>
@@ -1126,7 +1126,7 @@
         <x:v>스팀사용량 A</x:v>
       </x:c>
       <x:c r="C6" s="38" t="str">
-        <x:v>ton</x:v>
+        <x:v>t/h</x:v>
       </x:c>
       <x:c r="D6" s="38" t="str">
         <x:v>1시간</x:v>
@@ -1135,22 +1135,22 @@
         <x:v>범위 확인</x:v>
       </x:c>
       <x:c r="F6" s="38" t="n">
-        <x:v>0.2355</x:v>
+        <x:v>2.355</x:v>
       </x:c>
       <x:c r="G6" s="38" t="n">
-        <x:v>0.2684</x:v>
+        <x:v>2.684</x:v>
       </x:c>
       <x:c r="H6" s="38" t="n">
-        <x:v>0.2313</x:v>
+        <x:v>2.313</x:v>
       </x:c>
       <x:c r="I6" s="38" t="n">
-        <x:v>0.2734</x:v>
+        <x:v>2.734</x:v>
       </x:c>
       <x:c r="J6" s="38" t="n">
-        <x:v>0.2313</x:v>
+        <x:v>2.313</x:v>
       </x:c>
       <x:c r="K6" s="38" t="n">
-        <x:v>0.2734</x:v>
+        <x:v>2.734</x:v>
       </x:c>
       <x:c r="L6" s="42" t="str">
         <x:v>정상 P2.5~P97.5, 주의 P0.5~P2.5 또는 P97.5~P99.5, 이상은 그 밖 (정상 구간 경고+이상 약 5%)</x:v>
@@ -1164,7 +1164,7 @@
         <x:v>스팀사용량 B</x:v>
       </x:c>
       <x:c r="C7" s="38" t="str">
-        <x:v>ton</x:v>
+        <x:v>t/h</x:v>
       </x:c>
       <x:c r="D7" s="38" t="str">
         <x:v>1시간</x:v>
@@ -1173,22 +1173,22 @@
         <x:v>범위 확인</x:v>
       </x:c>
       <x:c r="F7" s="38" t="n">
-        <x:v>0.2356</x:v>
+        <x:v>2.356</x:v>
       </x:c>
       <x:c r="G7" s="38" t="n">
-        <x:v>0.2688</x:v>
+        <x:v>2.6879999999999997</x:v>
       </x:c>
       <x:c r="H7" s="38" t="n">
-        <x:v>0.2317</x:v>
+        <x:v>2.3169999999999997</x:v>
       </x:c>
       <x:c r="I7" s="38" t="n">
-        <x:v>0.2731</x:v>
+        <x:v>2.731</x:v>
       </x:c>
       <x:c r="J7" s="38" t="n">
-        <x:v>0.2317</x:v>
+        <x:v>2.3169999999999997</x:v>
       </x:c>
       <x:c r="K7" s="38" t="n">
-        <x:v>0.2731</x:v>
+        <x:v>2.731</x:v>
       </x:c>
       <x:c r="L7" s="42" t="str">
         <x:v>정상 P2.5~P97.5, 주의 P0.5~P2.5 또는 P97.5~P99.5, 이상은 그 밖 (정상 구간 경고+이상 약 5%)</x:v>
@@ -1202,7 +1202,7 @@
         <x:v>스팀사용량 C</x:v>
       </x:c>
       <x:c r="C8" s="38" t="str">
-        <x:v>ton</x:v>
+        <x:v>t/h</x:v>
       </x:c>
       <x:c r="D8" s="38" t="str">
         <x:v>1시간</x:v>
@@ -1211,22 +1211,22 @@
         <x:v>범위 확인</x:v>
       </x:c>
       <x:c r="F8" s="38" t="n">
-        <x:v>0.2351</x:v>
+        <x:v>2.351</x:v>
       </x:c>
       <x:c r="G8" s="38" t="n">
-        <x:v>0.2682</x:v>
+        <x:v>2.682</x:v>
       </x:c>
       <x:c r="H8" s="38" t="n">
-        <x:v>0.2304</x:v>
+        <x:v>2.304</x:v>
       </x:c>
       <x:c r="I8" s="38" t="n">
-        <x:v>0.2721</x:v>
+        <x:v>2.721</x:v>
       </x:c>
       <x:c r="J8" s="38" t="n">
-        <x:v>0.2304</x:v>
+        <x:v>2.304</x:v>
       </x:c>
       <x:c r="K8" s="38" t="n">
-        <x:v>0.2721</x:v>
+        <x:v>2.721</x:v>
       </x:c>
       <x:c r="L8" s="42" t="str">
         <x:v>정상 P2.5~P97.5, 주의 P0.5~P2.5 또는 P97.5~P99.5, 이상은 그 밖 (정상 구간 경고+이상 약 5%)</x:v>
@@ -1240,7 +1240,7 @@
         <x:v>스팀사용량 D</x:v>
       </x:c>
       <x:c r="C9" s="38" t="str">
-        <x:v>ton</x:v>
+        <x:v>t/h</x:v>
       </x:c>
       <x:c r="D9" s="38" t="str">
         <x:v>1시간</x:v>
@@ -1249,22 +1249,22 @@
         <x:v>범위 확인</x:v>
       </x:c>
       <x:c r="F9" s="38" t="n">
-        <x:v>0.2351</x:v>
+        <x:v>2.351</x:v>
       </x:c>
       <x:c r="G9" s="38" t="n">
-        <x:v>0.2682</x:v>
+        <x:v>2.682</x:v>
       </x:c>
       <x:c r="H9" s="38" t="n">
-        <x:v>0.2308</x:v>
+        <x:v>2.308</x:v>
       </x:c>
       <x:c r="I9" s="38" t="n">
-        <x:v>0.2733</x:v>
+        <x:v>2.7329999999999997</x:v>
       </x:c>
       <x:c r="J9" s="38" t="n">
-        <x:v>0.2308</x:v>
+        <x:v>2.308</x:v>
       </x:c>
       <x:c r="K9" s="38" t="n">
-        <x:v>0.2733</x:v>
+        <x:v>2.7329999999999997</x:v>
       </x:c>
       <x:c r="L9" s="42" t="str">
         <x:v>정상 P2.5~P97.5, 주의 P0.5~P2.5 또는 P97.5~P99.5, 이상은 그 밖 (정상 구간 경고+이상 약 5%)</x:v>
@@ -1278,7 +1278,7 @@
         <x:v>스팀사용량 E</x:v>
       </x:c>
       <x:c r="C10" s="38" t="str">
-        <x:v>ton</x:v>
+        <x:v>t/h</x:v>
       </x:c>
       <x:c r="D10" s="38" t="str">
         <x:v>1시간</x:v>
@@ -1287,22 +1287,22 @@
         <x:v>범위 확인</x:v>
       </x:c>
       <x:c r="F10" s="38" t="n">
-        <x:v>0.235</x:v>
+        <x:v>2.3499999999999996</x:v>
       </x:c>
       <x:c r="G10" s="38" t="n">
-        <x:v>0.2679</x:v>
+        <x:v>2.6790000000000003</x:v>
       </x:c>
       <x:c r="H10" s="38" t="n">
-        <x:v>0.2298</x:v>
+        <x:v>2.298</x:v>
       </x:c>
       <x:c r="I10" s="38" t="n">
-        <x:v>0.2726</x:v>
+        <x:v>2.726</x:v>
       </x:c>
       <x:c r="J10" s="38" t="n">
-        <x:v>0.2298</x:v>
+        <x:v>2.298</x:v>
       </x:c>
       <x:c r="K10" s="38" t="n">
-        <x:v>0.2726</x:v>
+        <x:v>2.726</x:v>
       </x:c>
       <x:c r="L10" s="42" t="str">
         <x:v>정상 P2.5~P97.5, 주의 P0.5~P2.5 또는 P97.5~P99.5, 이상은 그 밖 (정상 구간 경고+이상 약 5%)</x:v>
@@ -1316,7 +1316,7 @@
         <x:v>스팀사용량 F</x:v>
       </x:c>
       <x:c r="C11" s="38" t="str">
-        <x:v>ton</x:v>
+        <x:v>t/h</x:v>
       </x:c>
       <x:c r="D11" s="38" t="str">
         <x:v>1시간</x:v>
@@ -1325,22 +1325,22 @@
         <x:v>범위 확인</x:v>
       </x:c>
       <x:c r="F11" s="38" t="n">
-        <x:v>0.2353</x:v>
+        <x:v>2.353</x:v>
       </x:c>
       <x:c r="G11" s="38" t="n">
-        <x:v>0.2689</x:v>
+        <x:v>2.6889999999999996</x:v>
       </x:c>
       <x:c r="H11" s="38" t="n">
-        <x:v>0.2308</x:v>
+        <x:v>2.308</x:v>
       </x:c>
       <x:c r="I11" s="38" t="n">
-        <x:v>0.2737</x:v>
+        <x:v>2.737</x:v>
       </x:c>
       <x:c r="J11" s="38" t="n">
-        <x:v>0.2308</x:v>
+        <x:v>2.308</x:v>
       </x:c>
       <x:c r="K11" s="38" t="n">
-        <x:v>0.2737</x:v>
+        <x:v>2.737</x:v>
       </x:c>
       <x:c r="L11" s="42" t="str">
         <x:v>정상 P2.5~P97.5, 주의 P0.5~P2.5 또는 P97.5~P99.5, 이상은 그 밖 (정상 구간 경고+이상 약 5%)</x:v>

</xml_diff>